<commit_message>
Update chip report site 2026-08-19
</commit_message>
<xml_diff>
--- a/outputs/chip-report/台股盤後籌碼_2026-08-19.xlsx
+++ b/outputs/chip-report/台股盤後籌碼_2026-08-19.xlsx
@@ -823,10 +823,8 @@
       <c r="K19" s="9" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>官方端點延遲</t>
-        </is>
+      <c r="A20" s="6" t="n">
+        <v>762.6299999999974</v>
       </c>
       <c r="B20" s="6" t="n"/>
       <c r="C20" s="6" t="n"/>
@@ -855,7 +853,7 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>TWSE MI_5MINS_HIST 暫時逾時；不影響收盤、法人、信用交易與期選籌碼資料。</t>
+          <t>45,071.34 - 44,308.71；TWSE MI_5MINS_HIST</t>
         </is>
       </c>
       <c r="B22" s="7" t="n"/>
@@ -2131,7 +2129,7 @@
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
         <is>
-          <t>這是 2026-08-19 的盤後籌碼正式版：加權指數收 44,719.35 點、跌 589.33 點，盤中高低點官方端點暫時延遲，成交值約 8,902.70 億元；TWSE 信用交易統計已補回，融資金額餘額 5,481.90 億、較前一交易日增加 11.78 億，融券餘額 188,334 張、較前一交易日減少 16,121 張。TAIFEX 的外資(大小台)期貨未平倉依原表合併口徑 = TXF + MXF/4 + TMF/20，8/19 約為 -81,813，與結算比約 2,463、與前日增減約 1,051；主表 OP 欄位維持 BC-SC 與 BP-SP 的淨額口徑。</t>
+          <t>這是 2026-08-19 的盤後籌碼正式版：加權指數收 44,719.35 點、跌 589.33 點，盤中最高 45,071.34 點、最低 44,308.71 點，成交值約 8,902.70 億元；TWSE 信用交易統計已補回，融資金額餘額 5,481.90 億、較前一交易日增加 11.78 億，融券餘額 188,334 張、較前一交易日減少 16,121 張。TAIFEX 的外資(大小台)期貨未平倉依原表合併口徑 = TXF + MXF/4 + TMF/20，8/19 約為 -81,813，與結算比約 2,463、與前日增減約 1,051；主表 OP 欄位維持 BC-SC 與 BP-SP 的淨額口徑。</t>
         </is>
       </c>
     </row>

</xml_diff>